<commit_message>
Update with revisions from user testing
</commit_message>
<xml_diff>
--- a/memberData.xlsx
+++ b/memberData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madmarshall/Documents/medicaidOversightMap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41D0969E-D16E-834D-803A-C183E0A53347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05D49C01-D10A-A645-867C-61391597FED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2860" yWindow="660" windowWidth="28200" windowHeight="15760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="1620" windowWidth="21400" windowHeight="15760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ASTHO  Member (Agency) Accounts" sheetId="1" r:id="rId1"/>
@@ -716,9 +716,6 @@
     <t>0021</t>
   </si>
   <si>
-    <t>Kentucky Department for Public Health</t>
-  </si>
-  <si>
     <t>KY-DoH</t>
   </si>
   <si>
@@ -734,9 +731,6 @@
     <t>Frankfort</t>
   </si>
   <si>
-    <t>https://www.chfs.ky.gov/agencies/dph/Documents/KDPH_ORGChart_2024.pdf</t>
-  </si>
-  <si>
     <t>Friedlander, Eric</t>
   </si>
   <si>
@@ -1980,6 +1974,12 @@
   </si>
   <si>
     <t>Data Not Available</t>
+  </si>
+  <si>
+    <t>Kentucky Cabinet for Health and Family Services</t>
+  </si>
+  <si>
+    <t>https://www.chfs.ky.gov/services/Pages/search.aspx</t>
   </si>
 </sst>
 </file>
@@ -2059,7 +2059,7 @@
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="(Do Not Modify) Row Checksum"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="(Do Not Modify) Modified On"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Account Number"/>
-    <tableColumn id="22" xr3:uid="{9E5AA338-49A7-E544-84ED-578AEFA2CD30}" name="jurisdictionName" dataDxfId="0"/>
+    <tableColumn id="22" xr3:uid="{9E5AA338-49A7-E544-84ED-578AEFA2CD30}" name="jurisdictionName" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Account Name"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Governor Term Year"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Acronym"/>
@@ -2070,7 +2070,7 @@
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="S/THO Acting"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="S/THO Assistant"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="City"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Org Chart" dataDxfId="1"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Org Chart" dataDxfId="0"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Secretary of Health"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Population"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="PHAB Accreditation"/>
@@ -2437,7 +2437,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -2505,7 +2505,7 @@
         <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>24</v>
@@ -2564,7 +2564,7 @@
         <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>39</v>
@@ -2629,7 +2629,7 @@
         <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>53</v>
@@ -2685,7 +2685,7 @@
         <v>64</v>
       </c>
       <c r="E5" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>65</v>
@@ -2703,7 +2703,7 @@
         <v>67</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="M5" s="1" t="s">
         <v>68</v>
@@ -2747,7 +2747,7 @@
         <v>75</v>
       </c>
       <c r="E6" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>76</v>
@@ -2812,7 +2812,7 @@
         <v>86</v>
       </c>
       <c r="E7" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>87</v>
@@ -2871,7 +2871,7 @@
         <v>96</v>
       </c>
       <c r="E8" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>97</v>
@@ -2933,7 +2933,7 @@
         <v>105</v>
       </c>
       <c r="E9" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>106</v>
@@ -2995,7 +2995,7 @@
         <v>114</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>115</v>
@@ -3057,7 +3057,7 @@
         <v>124</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>125</v>
@@ -3119,7 +3119,7 @@
         <v>134</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>135</v>
@@ -3181,7 +3181,7 @@
         <v>144</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>145</v>
@@ -3240,7 +3240,7 @@
         <v>152</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>153</v>
@@ -3296,7 +3296,7 @@
         <v>163</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>164</v>
@@ -3349,7 +3349,7 @@
         <v>172</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>173</v>
@@ -3411,7 +3411,7 @@
         <v>181</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>182</v>
@@ -3473,7 +3473,7 @@
         <v>191</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>192</v>
@@ -3535,7 +3535,7 @@
         <v>201</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>202</v>
@@ -3597,7 +3597,7 @@
         <v>210</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>211</v>
@@ -3662,7 +3662,7 @@
         <v>221</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>222</v>
@@ -3724,16 +3724,16 @@
         <v>230</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>231</v>
+        <v>651</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>154</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>41</v>
@@ -3742,22 +3742,22 @@
         <v>137</v>
       </c>
       <c r="K22" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="L22" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="L22" s="1" t="s">
+      <c r="N22" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="N22" s="1" t="s">
+      <c r="O22" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="O22" s="1" t="s">
+      <c r="P22" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="Q22" s="1" t="s">
         <v>236</v>
-      </c>
-      <c r="P22" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="Q22" s="1" t="s">
-        <v>238</v>
       </c>
       <c r="R22" s="3">
         <v>4588372</v>
@@ -3777,28 +3777,28 @@
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C23" s="2">
         <v>45863.837233796301</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>41</v>
@@ -3807,19 +3807,19 @@
         <v>42</v>
       </c>
       <c r="K23" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="O23" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="N23" s="1" t="s">
+      <c r="P23" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="O23" s="1" t="s">
+      <c r="Q23" s="1" t="s">
         <v>246</v>
-      </c>
-      <c r="P23" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="Q23" s="1" t="s">
-        <v>248</v>
       </c>
       <c r="R23" s="3">
         <v>1405012</v>
@@ -3839,49 +3839,49 @@
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C24" s="2">
         <v>45894.698414351798</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J24" t="s">
+        <v>252</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="L24" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="K24" s="1" t="s">
+      <c r="N24" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="L24" s="1" t="s">
+      <c r="O24" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="N24" s="1" t="s">
+      <c r="P24" s="4" t="s">
         <v>257</v>
-      </c>
-      <c r="O24" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="P24" s="4" t="s">
-        <v>259</v>
       </c>
       <c r="R24" s="3">
         <v>6263220</v>
@@ -3901,28 +3901,28 @@
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C25" s="2">
         <v>45894.6550810185</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>41</v>
@@ -3931,19 +3931,19 @@
         <v>67</v>
       </c>
       <c r="K25" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="O25" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="N25" s="1" t="s">
+      <c r="P25" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="O25" s="1" t="s">
+      <c r="Q25" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="P25" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="Q25" s="1" t="s">
-        <v>269</v>
       </c>
       <c r="R25" s="3">
         <v>7136171</v>
@@ -3963,28 +3963,28 @@
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C26" s="2">
         <v>45894.698807870402</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>41</v>
@@ -3993,22 +3993,22 @@
         <v>67</v>
       </c>
       <c r="K26" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="N26" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L26" s="1" t="s">
+      <c r="O26" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="N26" s="1" t="s">
+      <c r="P26" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="O26" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="P26" s="4" t="s">
-        <v>279</v>
-      </c>
       <c r="Q26" s="1" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="R26" s="3">
         <v>10140459</v>
@@ -4028,28 +4028,28 @@
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C27" s="2">
         <v>45863.839803240699</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="G27" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>27</v>
@@ -4058,19 +4058,19 @@
         <v>67</v>
       </c>
       <c r="K27" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="N27" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="O27" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="N27" s="1" t="s">
+      <c r="P27" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="O27" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="P27" s="4" t="s">
-        <v>288</v>
-      </c>
       <c r="Q27" s="1" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="R27" s="3">
         <v>5793151</v>
@@ -4090,28 +4090,28 @@
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C28" s="2">
         <v>45863.8406944444</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>154</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>27</v>
@@ -4120,19 +4120,19 @@
         <v>78</v>
       </c>
       <c r="K28" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="N28" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="O28" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="N28" s="1" t="s">
+      <c r="P28" s="4" t="s">
         <v>295</v>
       </c>
-      <c r="O28" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="P28" s="4" t="s">
-        <v>297</v>
-      </c>
       <c r="Q28" s="1" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="R28" s="3">
         <v>2943045</v>
@@ -4152,28 +4152,28 @@
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C29" s="2">
         <v>45863.842407407399</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>54</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>27</v>
@@ -4182,16 +4182,16 @@
         <v>67</v>
       </c>
       <c r="K29" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="N29" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="O29" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="N29" s="1" t="s">
+      <c r="P29" s="4" t="s">
         <v>304</v>
-      </c>
-      <c r="O29" s="1" t="s">
-        <v>305</v>
-      </c>
-      <c r="P29" s="4" t="s">
-        <v>306</v>
       </c>
       <c r="R29" s="3">
         <v>6245466</v>
@@ -4211,28 +4211,28 @@
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C30" s="2">
         <v>45863.842951388899</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="G30" s="1" t="s">
         <v>54</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>41</v>
@@ -4241,16 +4241,16 @@
         <v>67</v>
       </c>
       <c r="K30" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="P30" s="4" t="s">
         <v>312</v>
       </c>
-      <c r="O30" s="1" t="s">
+      <c r="Q30" s="1" t="s">
         <v>313</v>
-      </c>
-      <c r="P30" s="4" t="s">
-        <v>314</v>
-      </c>
-      <c r="Q30" s="1" t="s">
-        <v>315</v>
       </c>
       <c r="R30" s="3">
         <v>1137233</v>
@@ -4270,28 +4270,28 @@
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C31" s="2">
         <v>45894.652962963002</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>41</v>
@@ -4300,19 +4300,19 @@
         <v>67</v>
       </c>
       <c r="K31" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="N31" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="O31" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="N31" s="1" t="s">
+      <c r="P31" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="O31" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="P31" s="4" t="s">
-        <v>324</v>
-      </c>
       <c r="Q31" s="1" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="R31" s="3">
         <v>2005465</v>
@@ -4332,49 +4332,49 @@
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C32" s="2">
         <v>45967.634143518502</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>41</v>
       </c>
       <c r="K32" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="N32" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="L32" s="1" t="s">
+      <c r="O32" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="N32" s="1" t="s">
+      <c r="P32" s="4" t="s">
         <v>332</v>
       </c>
-      <c r="O32" s="1" t="s">
+      <c r="Q32" s="1" t="s">
         <v>333</v>
-      </c>
-      <c r="P32" s="4" t="s">
-        <v>334</v>
-      </c>
-      <c r="Q32" s="1" t="s">
-        <v>335</v>
       </c>
       <c r="R32" s="3">
         <v>3267467</v>
@@ -4394,28 +4394,28 @@
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C33" s="2">
         <v>45863.852916666699</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="G33" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>41</v>
@@ -4424,19 +4424,19 @@
         <v>28</v>
       </c>
       <c r="K33" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="N33" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="O33" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="N33" s="1" t="s">
+      <c r="P33" s="4" t="s">
         <v>342</v>
       </c>
-      <c r="O33" s="1" t="s">
+      <c r="Q33" s="1" t="s">
         <v>343</v>
-      </c>
-      <c r="P33" s="4" t="s">
-        <v>344</v>
-      </c>
-      <c r="Q33" s="1" t="s">
-        <v>345</v>
       </c>
       <c r="R33" s="3">
         <v>1409032</v>
@@ -4456,28 +4456,28 @@
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C34" s="2">
         <v>45863.853518518503</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>628</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="E34" s="1" t="s">
-        <v>630</v>
-      </c>
-      <c r="F34" s="1" t="s">
+      <c r="H34" s="1" t="s">
         <v>349</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>351</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>27</v>
@@ -4486,19 +4486,19 @@
         <v>67</v>
       </c>
       <c r="M34" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="N34" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="O34" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="N34" s="1" t="s">
+      <c r="P34" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="O34" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="P34" s="4" t="s">
-        <v>355</v>
-      </c>
       <c r="Q34" s="1" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="R34" s="3">
         <v>9500851</v>
@@ -4518,28 +4518,28 @@
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C35" s="2">
         <v>45863.855405092603</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>27</v>
@@ -4548,22 +4548,22 @@
         <v>78</v>
       </c>
       <c r="K35" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="N35" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="L35" s="1" t="s">
+      <c r="O35" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="N35" s="1" t="s">
+      <c r="P35" s="4" t="s">
         <v>363</v>
       </c>
-      <c r="O35" s="1" t="s">
-        <v>364</v>
-      </c>
-      <c r="P35" s="4" t="s">
-        <v>365</v>
-      </c>
       <c r="Q35" s="1" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="R35" s="3">
         <v>2130256</v>
@@ -4583,28 +4583,28 @@
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C36" s="2">
         <v>45863.856504629599</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>27</v>
@@ -4613,16 +4613,16 @@
         <v>67</v>
       </c>
       <c r="K36" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="O36" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="N36" s="1" t="s">
+      <c r="P36" s="4" t="s">
         <v>372</v>
-      </c>
-      <c r="O36" s="1" t="s">
-        <v>373</v>
-      </c>
-      <c r="P36" s="4" t="s">
-        <v>374</v>
       </c>
       <c r="R36" s="3">
         <v>19867248</v>
@@ -4642,28 +4642,28 @@
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C37" s="2">
         <v>45863.856921296298</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>54</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>41</v>
@@ -4672,19 +4672,19 @@
         <v>67</v>
       </c>
       <c r="K37" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="N37" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L37" s="1" t="s">
+      <c r="O37" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="N37" s="1" t="s">
+      <c r="P37" s="4" t="s">
         <v>382</v>
-      </c>
-      <c r="O37" s="1" t="s">
-        <v>383</v>
-      </c>
-      <c r="P37" s="4" t="s">
-        <v>384</v>
       </c>
       <c r="R37" s="3">
         <v>11046024</v>
@@ -4704,28 +4704,28 @@
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C38" s="2">
         <v>45915.679270833301</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="G38" s="1" t="s">
         <v>54</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>27</v>
@@ -4734,19 +4734,19 @@
         <v>67</v>
       </c>
       <c r="K38" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="N38" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="O38" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="N38" s="1" t="s">
+      <c r="P38" s="4" t="s">
         <v>391</v>
       </c>
-      <c r="O38" s="1" t="s">
+      <c r="Q38" s="1" t="s">
         <v>392</v>
-      </c>
-      <c r="P38" s="4" t="s">
-        <v>393</v>
-      </c>
-      <c r="Q38" s="1" t="s">
-        <v>394</v>
       </c>
       <c r="R38" s="3">
         <v>796568</v>
@@ -4766,43 +4766,43 @@
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C39" s="2">
         <v>45923.543495370403</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="I39" s="1" t="s">
         <v>41</v>
       </c>
       <c r="K39" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="N39" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="O39" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="N39" s="1" t="s">
+      <c r="P39" s="4" t="s">
         <v>401</v>
-      </c>
-      <c r="O39" s="1" t="s">
-        <v>402</v>
-      </c>
-      <c r="P39" s="4" t="s">
-        <v>403</v>
       </c>
       <c r="S39" s="1" t="s">
         <v>48</v>
@@ -4819,28 +4819,28 @@
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C40" s="2">
         <v>45979.8848842593</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="G40" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="I40" s="1" t="s">
         <v>27</v>
@@ -4849,19 +4849,19 @@
         <v>67</v>
       </c>
       <c r="K40" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="N40" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="O40" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="N40" s="1" t="s">
+      <c r="P40" s="4" t="s">
         <v>410</v>
       </c>
-      <c r="O40" s="1" t="s">
-        <v>411</v>
-      </c>
-      <c r="P40" s="4" t="s">
-        <v>412</v>
-      </c>
       <c r="Q40" s="1" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="R40" s="3">
         <v>11883304</v>
@@ -4881,28 +4881,28 @@
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="C41" s="2">
         <v>45863.859097222201</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="G41" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>27</v>
@@ -4911,16 +4911,16 @@
         <v>42</v>
       </c>
       <c r="K41" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="N41" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="O41" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="N41" s="1" t="s">
+      <c r="P41" s="4" t="s">
         <v>419</v>
-      </c>
-      <c r="O41" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="P41" s="4" t="s">
-        <v>421</v>
       </c>
       <c r="R41" s="3">
         <v>4095393</v>
@@ -4940,28 +4940,28 @@
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C42" s="2">
         <v>45894.699074074102</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="G42" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>41</v>
@@ -4970,22 +4970,22 @@
         <v>67</v>
       </c>
       <c r="K42" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="L42" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="N42" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="L42" s="1" t="s">
+      <c r="O42" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="N42" s="1" t="s">
+      <c r="P42" s="4" t="s">
         <v>429</v>
       </c>
-      <c r="O42" s="1" t="s">
+      <c r="Q42" s="1" t="s">
         <v>430</v>
-      </c>
-      <c r="P42" s="4" t="s">
-        <v>431</v>
-      </c>
-      <c r="Q42" s="1" t="s">
-        <v>432</v>
       </c>
       <c r="R42" s="3">
         <v>4272371</v>
@@ -5002,28 +5002,28 @@
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C43" s="2">
         <v>45863.859930555598</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>27</v>
@@ -5032,19 +5032,19 @@
         <v>42</v>
       </c>
       <c r="K43" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="N43" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="O43" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="N43" s="1" t="s">
+      <c r="P43" s="4" t="s">
         <v>439</v>
       </c>
-      <c r="O43" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="P43" s="4" t="s">
-        <v>441</v>
-      </c>
       <c r="Q43" s="1" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="R43" s="3">
         <v>13078751</v>
@@ -5064,43 +5064,43 @@
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="C44" s="2">
         <v>45894.6547685185</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="G44" s="1" t="s">
         <v>54</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>56</v>
       </c>
       <c r="K44" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="N44" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="O44" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="N44" s="1" t="s">
+      <c r="P44" s="4" t="s">
         <v>448</v>
-      </c>
-      <c r="O44" s="1" t="s">
-        <v>449</v>
-      </c>
-      <c r="P44" s="4" t="s">
-        <v>450</v>
       </c>
       <c r="S44" s="1" t="s">
         <v>48</v>
@@ -5117,43 +5117,43 @@
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C45" s="2">
         <v>45978.801053240699</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>54</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>41</v>
       </c>
       <c r="K45" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="L45" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="N45" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="L45" s="1" t="s">
+      <c r="O45" s="1" t="s">
         <v>457</v>
-      </c>
-      <c r="N45" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="O45" s="1" t="s">
-        <v>459</v>
       </c>
       <c r="S45" s="1" t="s">
         <v>48</v>
@@ -5170,46 +5170,46 @@
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C46" s="2">
         <v>45932.7257986111</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="G46" s="1" t="s">
         <v>154</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="I46" s="1" t="s">
         <v>41</v>
       </c>
       <c r="K46" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="N46" s="1" t="s">
         <v>465</v>
       </c>
-      <c r="L46" s="1" t="s">
+      <c r="O46" s="1" t="s">
         <v>466</v>
       </c>
-      <c r="N46" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="O46" s="1" t="s">
-        <v>468</v>
-      </c>
       <c r="Q46" s="1" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="S46" s="1" t="s">
         <v>48</v>
@@ -5226,28 +5226,28 @@
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="C47" s="2">
         <v>45863.8605902778</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="I47" s="1" t="s">
         <v>41</v>
@@ -5256,19 +5256,19 @@
         <v>78</v>
       </c>
       <c r="K47" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="N47" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="O47" s="1" t="s">
         <v>474</v>
       </c>
-      <c r="N47" s="1" t="s">
+      <c r="P47" s="4" t="s">
         <v>475</v>
       </c>
-      <c r="O47" s="1" t="s">
+      <c r="Q47" s="1" t="s">
         <v>476</v>
-      </c>
-      <c r="P47" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="Q47" s="1" t="s">
-        <v>478</v>
       </c>
       <c r="R47" s="3">
         <v>1112308</v>
@@ -5288,28 +5288,28 @@
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="C48" s="2">
         <v>45863.860983796301</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="I48" s="1" t="s">
         <v>27</v>
@@ -5318,22 +5318,22 @@
         <v>78</v>
       </c>
       <c r="L48" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="M48" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="N48" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="M48" s="1" t="s">
+      <c r="O48" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="N48" s="1" t="s">
+      <c r="P48" s="4" t="s">
         <v>486</v>
       </c>
-      <c r="O48" s="1" t="s">
-        <v>487</v>
-      </c>
-      <c r="P48" s="4" t="s">
-        <v>488</v>
-      </c>
       <c r="Q48" s="1" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="R48" s="3">
         <v>5478831</v>
@@ -5353,28 +5353,28 @@
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="C49" s="2">
         <v>45863.861412036997</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="I49" s="1" t="s">
         <v>27</v>
@@ -5383,19 +5383,19 @@
         <v>28</v>
       </c>
       <c r="K49" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="N49" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="O49" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="N49" s="1" t="s">
+      <c r="P49" s="4" t="s">
         <v>495</v>
       </c>
-      <c r="O49" s="1" t="s">
-        <v>496</v>
-      </c>
-      <c r="P49" s="4" t="s">
-        <v>497</v>
-      </c>
       <c r="Q49" s="1" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="R49" s="3">
         <v>924669</v>
@@ -5415,28 +5415,28 @@
     </row>
     <row r="50" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C50" s="2">
         <v>45959.7264699074</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="G50" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="I50" s="1" t="s">
         <v>27</v>
@@ -5445,13 +5445,13 @@
         <v>42</v>
       </c>
       <c r="K50" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="N50" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="O50" s="1" t="s">
         <v>503</v>
-      </c>
-      <c r="N50" s="1" t="s">
-        <v>504</v>
-      </c>
-      <c r="O50" s="1" t="s">
-        <v>505</v>
       </c>
       <c r="R50" s="3">
         <v>7227750</v>
@@ -5471,46 +5471,46 @@
     </row>
     <row r="51" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C51" s="2">
         <v>45863.863425925898</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="G51" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="I51" s="1" t="s">
         <v>27</v>
       </c>
       <c r="K51" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="N51" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="O51" s="1" t="s">
         <v>511</v>
       </c>
-      <c r="N51" s="1" t="s">
+      <c r="P51" s="4" t="s">
         <v>512</v>
       </c>
-      <c r="O51" s="1" t="s">
+      <c r="Q51" s="1" t="s">
         <v>513</v>
-      </c>
-      <c r="P51" s="4" t="s">
-        <v>514</v>
-      </c>
-      <c r="Q51" s="1" t="s">
-        <v>515</v>
       </c>
       <c r="R51" s="3">
         <v>31290831</v>
@@ -5530,46 +5530,46 @@
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="C52" s="2">
         <v>45839.724166666703</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="G52" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="I52" s="1" t="s">
         <v>56</v>
       </c>
       <c r="K52" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="N52" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="O52" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="N52" s="1" t="s">
+      <c r="P52" s="4" t="s">
         <v>522</v>
       </c>
-      <c r="O52" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="P52" s="4" t="s">
-        <v>524</v>
-      </c>
       <c r="Q52" s="1" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="S52" s="1" t="s">
         <v>48</v>
@@ -5586,28 +5586,28 @@
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C53" s="2">
         <v>45957.780775462998</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>54</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="I53" s="1" t="s">
         <v>27</v>
@@ -5616,19 +5616,19 @@
         <v>67</v>
       </c>
       <c r="K53" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="N53" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="O53" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="N53" s="1" t="s">
+      <c r="P53" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="Q53" s="1" t="s">
         <v>531</v>
-      </c>
-      <c r="O53" s="1" t="s">
-        <v>532</v>
-      </c>
-      <c r="P53" s="4" t="s">
-        <v>593</v>
-      </c>
-      <c r="Q53" s="1" t="s">
-        <v>533</v>
       </c>
       <c r="R53" s="3">
         <v>3503613</v>
@@ -5648,28 +5648,28 @@
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C54" s="2">
         <v>45944.531030092599</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="G54" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="I54" s="1" t="s">
         <v>41</v>
@@ -5678,19 +5678,19 @@
         <v>78</v>
       </c>
       <c r="K54" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="N54" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="O54" s="1" t="s">
         <v>539</v>
       </c>
-      <c r="N54" s="1" t="s">
+      <c r="P54" s="4" t="s">
         <v>540</v>
       </c>
-      <c r="O54" s="1" t="s">
+      <c r="Q54" s="1" t="s">
         <v>541</v>
-      </c>
-      <c r="P54" s="4" t="s">
-        <v>542</v>
-      </c>
-      <c r="Q54" s="1" t="s">
-        <v>543</v>
       </c>
       <c r="R54" s="3">
         <v>648493</v>
@@ -5710,28 +5710,28 @@
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="C55" s="2">
         <v>45894.698101851798</v>
       </c>
       <c r="D55" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>647</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="H55" s="1" t="s">
         <v>546</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>649</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>548</v>
       </c>
       <c r="I55" s="1" t="s">
         <v>27</v>
@@ -5740,19 +5740,19 @@
         <v>28</v>
       </c>
       <c r="K55" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="N55" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="O55" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="N55" s="1" t="s">
+      <c r="P55" s="4" t="s">
         <v>550</v>
       </c>
-      <c r="O55" s="1" t="s">
+      <c r="Q55" s="1" t="s">
         <v>551</v>
-      </c>
-      <c r="P55" s="4" t="s">
-        <v>552</v>
-      </c>
-      <c r="Q55" s="1" t="s">
-        <v>553</v>
       </c>
       <c r="R55" s="3">
         <v>8535519</v>
@@ -5772,28 +5772,28 @@
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="C56" s="2">
         <v>45894.668194444399</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>129</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>54</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="I56" s="1" t="s">
         <v>27</v>
@@ -5802,19 +5802,19 @@
         <v>67</v>
       </c>
       <c r="K56" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="N56" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="O56" s="1" t="s">
         <v>559</v>
       </c>
-      <c r="N56" s="1" t="s">
+      <c r="P56" s="4" t="s">
         <v>560</v>
       </c>
-      <c r="O56" s="1" t="s">
-        <v>561</v>
-      </c>
-      <c r="P56" s="4" t="s">
-        <v>562</v>
-      </c>
       <c r="Q56" s="1" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="R56" s="3">
         <v>7614893</v>
@@ -5834,28 +5834,28 @@
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C57" s="2">
         <v>45894.632835648103</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>54</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="I57" s="1" t="s">
         <v>41</v>
@@ -5864,16 +5864,16 @@
         <v>67</v>
       </c>
       <c r="M57" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="N57" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="O57" s="1" t="s">
         <v>568</v>
       </c>
-      <c r="N57" s="1" t="s">
+      <c r="P57" s="4" t="s">
         <v>569</v>
-      </c>
-      <c r="O57" s="1" t="s">
-        <v>570</v>
-      </c>
-      <c r="P57" s="4" t="s">
-        <v>571</v>
       </c>
       <c r="R57" s="3">
         <v>1792147</v>
@@ -5893,28 +5893,28 @@
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C58" s="2">
         <v>45894.697719907403</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="I58" s="1" t="s">
         <v>41</v>
@@ -5923,19 +5923,19 @@
         <v>67</v>
       </c>
       <c r="K58" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="N58" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="O58" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="N58" s="1" t="s">
+      <c r="P58" s="4" t="s">
         <v>578</v>
       </c>
-      <c r="O58" s="1" t="s">
+      <c r="Q58" s="1" t="s">
         <v>579</v>
-      </c>
-      <c r="P58" s="4" t="s">
-        <v>580</v>
-      </c>
-      <c r="Q58" s="1" t="s">
-        <v>581</v>
       </c>
       <c r="R58" s="3">
         <v>5822434</v>
@@ -5955,28 +5955,28 @@
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C59" s="2">
         <v>45894.668796296297</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>25</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="I59" s="1" t="s">
         <v>41</v>
@@ -5985,19 +5985,19 @@
         <v>42</v>
       </c>
       <c r="K59" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="L59" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="O59" s="1" t="s">
         <v>587</v>
       </c>
-      <c r="L59" s="1" t="s">
+      <c r="P59" s="4" t="s">
         <v>588</v>
       </c>
-      <c r="O59" s="1" t="s">
+      <c r="Q59" s="1" t="s">
         <v>589</v>
-      </c>
-      <c r="P59" s="4" t="s">
-        <v>590</v>
-      </c>
-      <c r="Q59" s="1" t="s">
-        <v>591</v>
       </c>
       <c r="R59" s="3">
         <v>578759</v>
@@ -6069,44 +6069,43 @@
     <hyperlink ref="P19" r:id="rId17" xr:uid="{0A2FA18A-514A-4366-A4EC-51C1EECDD28E}"/>
     <hyperlink ref="P20" r:id="rId18" xr:uid="{E07E0A34-F6A5-4745-AEEF-3E1D7D81F532}"/>
     <hyperlink ref="P21" r:id="rId19" xr:uid="{6681FC06-699D-4557-A261-080A7381AFE8}"/>
-    <hyperlink ref="P22" r:id="rId20" xr:uid="{2619FDDF-555F-42A3-87B5-8A609128F3C8}"/>
-    <hyperlink ref="P23" r:id="rId21" xr:uid="{94341740-42F6-49C7-AAFE-AF32E4009868}"/>
-    <hyperlink ref="P24" r:id="rId22" xr:uid="{EE469778-AF12-44E8-9820-50B413511AA6}"/>
-    <hyperlink ref="P25" r:id="rId23" xr:uid="{4B87F942-D74D-4166-970E-F5E5748AC8FB}"/>
-    <hyperlink ref="P26" r:id="rId24" xr:uid="{0993A219-6BF1-4317-A442-00036BB4FC92}"/>
-    <hyperlink ref="P27" r:id="rId25" xr:uid="{1CD243D6-2B7E-4943-B0B2-9FF6A7F4DAD6}"/>
-    <hyperlink ref="P28" r:id="rId26" xr:uid="{41EFFD08-4853-4A26-884E-1DF33B76A091}"/>
-    <hyperlink ref="P29" r:id="rId27" xr:uid="{F467495C-2D06-460C-8031-D4DFC78B4B10}"/>
-    <hyperlink ref="P30" r:id="rId28" xr:uid="{3A81479C-E1E5-40B7-8789-6A2840D4AFC8}"/>
-    <hyperlink ref="P31" r:id="rId29" xr:uid="{1F619310-E327-4DD2-8A71-6E446F73F006}"/>
-    <hyperlink ref="P32" r:id="rId30" xr:uid="{2681B774-ABCC-4F44-B952-8DFDD89DCEBB}"/>
-    <hyperlink ref="P33" r:id="rId31" xr:uid="{FC5E12E2-FD76-4325-8EAD-7C4DDA76A065}"/>
-    <hyperlink ref="P34" r:id="rId32" xr:uid="{7E2A3350-D14F-4A06-951E-30ACE91438AD}"/>
-    <hyperlink ref="P35" r:id="rId33" xr:uid="{83082298-87E6-4F3B-9D14-AB47400E721E}"/>
-    <hyperlink ref="P36" r:id="rId34" xr:uid="{FA22572E-5860-496A-AC81-405711971BED}"/>
-    <hyperlink ref="P37" r:id="rId35" xr:uid="{FF83F8F9-C8A9-4C9A-8CE4-FBCC1BAD81F4}"/>
-    <hyperlink ref="P38" r:id="rId36" xr:uid="{A5D25D1C-155D-44F2-912A-08A4233D68C7}"/>
-    <hyperlink ref="P39" r:id="rId37" xr:uid="{11DB7D3D-A850-4079-A7E0-0E6C2566A9BA}"/>
-    <hyperlink ref="P40" r:id="rId38" xr:uid="{465ED70A-6593-48EC-A551-2C2BF30A4C8D}"/>
-    <hyperlink ref="P41" r:id="rId39" xr:uid="{54894BC2-584D-42CA-B554-32AA68974C32}"/>
-    <hyperlink ref="P42" r:id="rId40" xr:uid="{98E1F1AD-7866-4703-B8AE-A769512E3AB2}"/>
-    <hyperlink ref="P43" r:id="rId41" xr:uid="{D374230A-1E43-4A39-AF8C-EB35DB90FFB3}"/>
-    <hyperlink ref="P44" r:id="rId42" xr:uid="{113308A8-CF5E-4FC5-BE08-A179B8875873}"/>
-    <hyperlink ref="P47" r:id="rId43" xr:uid="{48DB851A-A65D-4C19-9DA6-C08E306672B0}"/>
-    <hyperlink ref="P48" r:id="rId44" xr:uid="{AB47AAE3-F3FC-4F4E-8B96-AFCD45801C87}"/>
-    <hyperlink ref="P49" r:id="rId45" xr:uid="{94D77222-2596-443F-A198-D1ACA09491C2}"/>
-    <hyperlink ref="P51" r:id="rId46" xr:uid="{31F276A7-B8A7-4948-AD8C-2B424176A3F5}"/>
-    <hyperlink ref="P52" r:id="rId47" xr:uid="{3E3BD377-1012-48DD-9D8E-EE9BDAEC6E1C}"/>
-    <hyperlink ref="P54" r:id="rId48" xr:uid="{9EDFD108-00F8-4944-853D-9CF322D9F19C}"/>
-    <hyperlink ref="P55" r:id="rId49" xr:uid="{D7B0DACD-5FD1-4346-B4E7-958EFDE6DA7C}"/>
-    <hyperlink ref="P56" r:id="rId50" xr:uid="{55EB6149-0908-4B53-A043-978695B6AFF2}"/>
-    <hyperlink ref="P57" r:id="rId51" xr:uid="{566E4284-EA29-42AE-ADF0-6D11CA2D7918}"/>
-    <hyperlink ref="P58" r:id="rId52" xr:uid="{1F555AFE-78CF-4F3C-9D4D-8A9484A22E05}"/>
-    <hyperlink ref="P59" r:id="rId53" xr:uid="{A07AD047-9BF8-4A20-B9F9-4A6749EA616A}"/>
+    <hyperlink ref="P23" r:id="rId20" xr:uid="{94341740-42F6-49C7-AAFE-AF32E4009868}"/>
+    <hyperlink ref="P24" r:id="rId21" xr:uid="{EE469778-AF12-44E8-9820-50B413511AA6}"/>
+    <hyperlink ref="P25" r:id="rId22" xr:uid="{4B87F942-D74D-4166-970E-F5E5748AC8FB}"/>
+    <hyperlink ref="P26" r:id="rId23" xr:uid="{0993A219-6BF1-4317-A442-00036BB4FC92}"/>
+    <hyperlink ref="P27" r:id="rId24" xr:uid="{1CD243D6-2B7E-4943-B0B2-9FF6A7F4DAD6}"/>
+    <hyperlink ref="P28" r:id="rId25" xr:uid="{41EFFD08-4853-4A26-884E-1DF33B76A091}"/>
+    <hyperlink ref="P29" r:id="rId26" xr:uid="{F467495C-2D06-460C-8031-D4DFC78B4B10}"/>
+    <hyperlink ref="P30" r:id="rId27" xr:uid="{3A81479C-E1E5-40B7-8789-6A2840D4AFC8}"/>
+    <hyperlink ref="P31" r:id="rId28" xr:uid="{1F619310-E327-4DD2-8A71-6E446F73F006}"/>
+    <hyperlink ref="P32" r:id="rId29" xr:uid="{2681B774-ABCC-4F44-B952-8DFDD89DCEBB}"/>
+    <hyperlink ref="P33" r:id="rId30" xr:uid="{FC5E12E2-FD76-4325-8EAD-7C4DDA76A065}"/>
+    <hyperlink ref="P34" r:id="rId31" xr:uid="{7E2A3350-D14F-4A06-951E-30ACE91438AD}"/>
+    <hyperlink ref="P35" r:id="rId32" xr:uid="{83082298-87E6-4F3B-9D14-AB47400E721E}"/>
+    <hyperlink ref="P36" r:id="rId33" xr:uid="{FA22572E-5860-496A-AC81-405711971BED}"/>
+    <hyperlink ref="P37" r:id="rId34" xr:uid="{FF83F8F9-C8A9-4C9A-8CE4-FBCC1BAD81F4}"/>
+    <hyperlink ref="P38" r:id="rId35" xr:uid="{A5D25D1C-155D-44F2-912A-08A4233D68C7}"/>
+    <hyperlink ref="P39" r:id="rId36" xr:uid="{11DB7D3D-A850-4079-A7E0-0E6C2566A9BA}"/>
+    <hyperlink ref="P40" r:id="rId37" xr:uid="{465ED70A-6593-48EC-A551-2C2BF30A4C8D}"/>
+    <hyperlink ref="P41" r:id="rId38" xr:uid="{54894BC2-584D-42CA-B554-32AA68974C32}"/>
+    <hyperlink ref="P42" r:id="rId39" xr:uid="{98E1F1AD-7866-4703-B8AE-A769512E3AB2}"/>
+    <hyperlink ref="P43" r:id="rId40" xr:uid="{D374230A-1E43-4A39-AF8C-EB35DB90FFB3}"/>
+    <hyperlink ref="P44" r:id="rId41" xr:uid="{113308A8-CF5E-4FC5-BE08-A179B8875873}"/>
+    <hyperlink ref="P47" r:id="rId42" xr:uid="{48DB851A-A65D-4C19-9DA6-C08E306672B0}"/>
+    <hyperlink ref="P48" r:id="rId43" xr:uid="{AB47AAE3-F3FC-4F4E-8B96-AFCD45801C87}"/>
+    <hyperlink ref="P49" r:id="rId44" xr:uid="{94D77222-2596-443F-A198-D1ACA09491C2}"/>
+    <hyperlink ref="P51" r:id="rId45" xr:uid="{31F276A7-B8A7-4948-AD8C-2B424176A3F5}"/>
+    <hyperlink ref="P52" r:id="rId46" xr:uid="{3E3BD377-1012-48DD-9D8E-EE9BDAEC6E1C}"/>
+    <hyperlink ref="P54" r:id="rId47" xr:uid="{9EDFD108-00F8-4944-853D-9CF322D9F19C}"/>
+    <hyperlink ref="P55" r:id="rId48" xr:uid="{D7B0DACD-5FD1-4346-B4E7-958EFDE6DA7C}"/>
+    <hyperlink ref="P56" r:id="rId49" xr:uid="{55EB6149-0908-4B53-A043-978695B6AFF2}"/>
+    <hyperlink ref="P57" r:id="rId50" xr:uid="{566E4284-EA29-42AE-ADF0-6D11CA2D7918}"/>
+    <hyperlink ref="P58" r:id="rId51" xr:uid="{1F555AFE-78CF-4F3C-9D4D-8A9484A22E05}"/>
+    <hyperlink ref="P59" r:id="rId52" xr:uid="{A07AD047-9BF8-4A20-B9F9-4A6749EA616A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId54"/>
+    <tablePart r:id="rId53"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -6137,7 +6136,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>